<commit_message>
CAR Varones: codigos de lamina del metrado cambiados a los DPLV del juego final (solo textos, valores iguales)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/insumos/metrados_vigentes/METRADO_DRENAJE_PLUVIAL_CAR_VARONES.xlsx
+++ b/insumos/metrados_vigentes/METRADO_DRENAJE_PLUVIAL_CAR_VARONES.xlsx
@@ -1861,7 +1861,7 @@
     <t>CUNETAS - ACORTAMIENTO EN LA LLEGADA AL COLECTOR PLUVIAL FRONTAL</t>
   </si>
   <si>
-    <t>Las cunetas estan dibujadas hasta la franja exterior del frente. El colector pluvial frontal ocupa esa franja, por lo que cada cuneta termina en la cara del muro lado predio del colector (ventana de empalme, lamina DP-06C) o en el muro norte de la caja de llegada CL del Hogar de Refugio (Eje 01, lamina DP-07). El tramo que caia dentro del colector se descuenta de la longitud de la cuneta en todas las hojas de este metrado (concreto, encofrado, acero, curado, rejillas, juntas, movimiento de tierras).</t>
+    <t>Las cunetas estan dibujadas hasta la franja exterior del frente. El colector pluvial frontal ocupa esa franja, por lo que cada cuneta termina en la cara del muro lado predio del colector (ventana de empalme, lamina DPLV-24) o en el muro norte de la caja de llegada CL del Hogar de Refugio (Eje 01, lamina DPLV-25). El tramo que caia dentro del colector se descuenta de la longitud de la cuneta en todas las hojas de este metrado (concreto, encofrado, acero, curado, rejillas, juntas, movimiento de tierras).</t>
   </si>
   <si>
     <t>CUNETA</t>
@@ -1885,7 +1885,7 @@
     <t>muro norte de la caja CL</t>
   </si>
   <si>
-    <t>Lamina DP-01 del colector (planta: tramo de cuneta que se descuenta) y memoria de calculo del colector, hoja CUNETAS</t>
+    <t>Lamina DPLV-17 del colector (planta: tramo de cuneta que se descuenta) y memoria de calculo del colector, hoja CUNETAS</t>
   </si>
   <si>
     <t>muro del colector (ventana)</t>
@@ -2023,7 +2023,7 @@
     <t>COLECTOR PLUVIAL FRONTAL - PARAMETROS DE METRADO</t>
   </si>
   <si>
-    <t>Tramo CAR Varones (CUI 2705619), empalme con la caja de llegada CL del colector del Hogar de Refugio Temporal (CUI 2675514). Valores tomados de los planos DP-01 a DP-08, DA-01 a DA-03 y DD-01 a DD-04 y de la memoria de calculo del colector. Celda amarilla = dato; verde = formula.</t>
+    <t>Tramo CAR Varones (CUI 2705619), empalme con la caja de llegada CL del colector del Hogar de Refugio Temporal (CUI 2675514). Valores tomados de las laminas DPLV-17 a DPLV-30 y de la memoria de calculo del colector. Celda amarilla = dato; verde = formula.</t>
   </si>
   <si>
     <t>PARAMETRO</t>
@@ -2035,37 +2035,37 @@
     <t>Ancho interior del colector b</t>
   </si>
   <si>
-    <t>Lamina DP-04 (secciones); memoria de calculo, hoja DATOS</t>
+    <t>Laminas DPLV-21 y DPLV-22 (secciones); memoria de calculo, hoja DATOS</t>
   </si>
   <si>
     <t>Espesor de muros</t>
   </si>
   <si>
-    <t>Lamina DP-04; memoria, hoja ESTRUCTURAL</t>
+    <t>Laminas DPLV-21 y DPLV-22; memoria, hoja ESTRUCTURAL</t>
   </si>
   <si>
     <t>Espesor de losa de fondo</t>
   </si>
   <si>
-    <t>Lamina DP-04</t>
+    <t>Laminas DPLV-21 y DPLV-22</t>
   </si>
   <si>
     <t>Espesor de losa superior (tramo normal)</t>
   </si>
   <si>
-    <t>Lamina DP-04 (secciones S-02 a S-08)</t>
+    <t>Laminas DPLV-21 y DPLV-22 (secciones S-02 a S-08)</t>
   </si>
   <si>
     <t>Espesor de losa superior (cruce de camiones cisterna)</t>
   </si>
   <si>
-    <t>Lamina DP-04 (seccion S-01); memoria, hoja ESTRUCTURAL (carga HL-93)</t>
+    <t>Lamina DPLV-21 (seccion S-01); memoria, hoja ESTRUCTURAL (carga HL-93)</t>
   </si>
   <si>
     <t>Espesor de solado</t>
   </si>
   <si>
-    <t>Lamina DP-04 y DA-02</t>
+    <t>Laminas DPLV-21 y DPLV-22</t>
   </si>
   <si>
     <t>Nivel de piso terminado del frente (cara superior de la losa)</t>
@@ -2074,19 +2074,19 @@
     <t>msnm</t>
   </si>
   <si>
-    <t>Lamina DP-02 (perfil) y plano de arquitectura (+261.15)</t>
+    <t>Lamina DPLV-18 (perfil) y plano de arquitectura (+261.15)</t>
   </si>
   <si>
     <t>Sobreancho de excavacion a cada lado del colector</t>
   </si>
   <si>
-    <t>Lamina DA-01: zanja de 1.40 m (0.90 + 2 x 0.25)</t>
+    <t>Laminas DPLV-21 y DPLV-22: zanja de 1.40 m (0.90 + 2 x 0.25)</t>
   </si>
   <si>
     <t>Franja de relleno de nivelacion del retiro, lado via</t>
   </si>
   <si>
-    <t>Lamina DA-01, nota 2</t>
+    <t>Laminas DPLV-21 y DPLV-22</t>
   </si>
   <si>
     <t>Recubrimiento del acero</t>
@@ -2122,7 +2122,7 @@
     <t>Ganchos de cierre del marco (2 x 0.15)</t>
   </si>
   <si>
-    <t>Lamina DP-08, cuadro de doblado</t>
+    <t>Laminas DPLV-21 y DPLV-22, armadura</t>
   </si>
   <si>
     <t>Igual a PARAMETROS!B16 de esta planilla</t>
@@ -2131,13 +2131,13 @@
     <t>Espaciamiento de marcos en tramo normal</t>
   </si>
   <si>
-    <t>Lamina DP-04 y DP-08</t>
+    <t>Laminas DPLV-21 y DPLV-22</t>
   </si>
   <si>
     <t>Espaciamiento de marcos en el cruce de camiones</t>
   </si>
   <si>
-    <t>Lamina DP-04 (seccion S-01) y DP-08</t>
+    <t>Lamina DPLV-21 (seccion S-01)</t>
   </si>
   <si>
     <t>Espaciamiento de barras longitudinales (tramo normal)</t>
@@ -2149,13 +2149,13 @@
     <t>Numero de registros de limpieza con tapa</t>
   </si>
   <si>
-    <t>Lamina DP-01 (RV-01 a RV-11), todos en la losa del colector; hoja COLECTOR REGISTROS Y TAPAS</t>
+    <t>Lamina DPLV-17 (RV-01 a RV-11), todos en la losa del colector; hoja COLECTOR REGISTROS Y TAPAS</t>
   </si>
   <si>
     <t>Lado de la tapa de concreto</t>
   </si>
   <si>
-    <t>Lamina DP-06B</t>
+    <t>Lamina DPLV-23</t>
   </si>
   <si>
     <t>Espesor de la tapa</t>
@@ -2170,31 +2170,31 @@
     <t>Cota de fondo del colector en el arranque (0+000)</t>
   </si>
   <si>
-    <t>Lamina DP-02; memoria, hoja PERFIL_FLUJO</t>
+    <t>Lamina DPLV-18; memoria, hoja PERFIL_FLUJO</t>
   </si>
   <si>
     <t>Cota de fondo del colector en la llegada a la CL (0+105.29)</t>
   </si>
   <si>
-    <t>Lamina DP-02 y DP-07; memoria, hoja EMPALME_CL</t>
+    <t>Laminas DPLV-18 y DPLV-25; memoria, hoja EMPALME_CL</t>
   </si>
   <si>
     <t>Espaciamiento de juntas de dilatacion</t>
   </si>
   <si>
-    <t>Lamina DP-01, nota; DP-02</t>
+    <t>Lamina DPLV-17, nota; DPLV-18</t>
   </si>
   <si>
     <t>Altura interior maxima del colector (para el perimetro de la junta)</t>
   </si>
   <si>
-    <t>Lamina DP-02 (perfil): llegada a la CL</t>
+    <t>Lamina DPLV-18 (perfil): llegada a la CL</t>
   </si>
   <si>
     <t>Progresiva final (cara este de la caja CL)</t>
   </si>
   <si>
-    <t>Lamina DP-01</t>
+    <t>Lamina DPLV-17</t>
   </si>
   <si>
     <t>Progresiva del quiebre (inicio del tramo de empalme)</t>
@@ -2203,13 +2203,13 @@
     <t>Ancho exterior del muro este de la caja CL (contacto con el colector)</t>
   </si>
   <si>
-    <t>Lamina DP-07</t>
+    <t>Lamina DPLV-25</t>
   </si>
   <si>
     <t>COLECTOR PLUVIAL FRONTAL - METRADO DE MOVIMIENTO DE TIERRAS</t>
   </si>
   <si>
-    <t>Criterio (lamina DA-01): LIMPIEZA Y TRAZO = ancho de zanja x L.  EXCAVACION = ancho de zanja x Hz x L, con Hz = terreno existente (topografia) - fondo del solado.  REFINE = (ancho exterior + 0.10) x L (fondo del solado).  RELLENO LATERAL = 2 x sobreancho x Hz x L.  RELLENO FRANJA = 1.00 x (NPT - terreno) x L (nivelacion del retiro lado via).  h y Hz son valores medios ponderados del tramo (perfil DP-02 y topografia); el detalle cada 2.00 m esta en la memoria de calculo.</t>
+    <t>Criterio (laminas DPLV-21 y DPLV-22): LIMPIEZA Y TRAZO = ancho de zanja x L.  EXCAVACION = ancho de zanja x Hz x L, con Hz = terreno existente (topografia) - fondo del solado.  REFINE = (ancho exterior + 0.10) x L (fondo del solado).  RELLENO LATERAL = 2 x sobreancho x Hz x L.  RELLENO FRANJA = 1.00 x (NPT - terreno) x L (nivelacion del retiro lado via).  h y Hz son valores medios ponderados del tramo (perfil DPLV-18 y topografia); el detalle cada 2.00 m esta en la memoria de calculo.</t>
   </si>
   <si>
     <t>ZONA</t>
@@ -2266,7 +2266,7 @@
     <t>0+006.08</t>
   </si>
   <si>
-    <t>DP-01 (planta), DP-02 (perfil: fondo y terreno), DP-04 (seccion), DA-01 (criterio)</t>
+    <t>DPLV-17 (planta), DPLV-18 (perfil: fondo y terreno), DPLV-21 y DPLV-22 (seccion y criterio)</t>
   </si>
   <si>
     <t>tramo normal</t>
@@ -2311,7 +2311,7 @@
     <t>COLECTOR PLUVIAL FRONTAL - METRADO DE CONCRETO SIMPLE Y ARMADO</t>
   </si>
   <si>
-    <t>Criterio (lamina DA-02): SOLADO = (ancho exterior + 0.10) x L.  LOSA DE FONDO = ancho exterior x e fondo x L.  MUROS = 2 x e muro x h x L.  LOSA SUPERIOR = ancho exterior x e losa x L.  ACABADO = ancho exterior x L (losa superior frotachada y brunada).  CURADO = 2 caras interiores de muros (2 x h x L) + fondo interior (b x L) + losa superior (ancho exterior x L), igual al criterio de la hoja METRADO DE CURADO.</t>
+    <t>Criterio (laminas DPLV-21 y DPLV-22): SOLADO = (ancho exterior + 0.10) x L.  LOSA DE FONDO = ancho exterior x e fondo x L.  MUROS = 2 x e muro x h x L.  LOSA SUPERIOR = ancho exterior x e losa x L.  ACABADO = ancho exterior x L (losa superior frotachada y brunada).  CURADO = 2 caras interiores de muros (2 x h x L) + fondo interior (b x L) + losa superior (ancho exterior x L), igual al criterio de la hoja METRADO DE CURADO.</t>
   </si>
   <si>
     <t>ANCHO EXT. (m)</t>
@@ -2335,7 +2335,7 @@
     <t>CURADO (m2)</t>
   </si>
   <si>
-    <t>DP-04 (secciones), DP-02 (h por tramo), DA-02 (areas por metro)</t>
+    <t>DPLV-21 y DPLV-22 (secciones y areas por metro), DPLV-18 (h por tramo)</t>
   </si>
   <si>
     <t>TOTAL COLECTOR (tramos)</t>
@@ -2365,7 +2365,7 @@
     <t>perimetro x seccion</t>
   </si>
   <si>
-    <t>DP-06B</t>
+    <t>DPLV-23</t>
   </si>
   <si>
     <t>TOTAL REGISTROS</t>
@@ -2392,7 +2392,7 @@
     <t>COLECTOR PLUVIAL FRONTAL - METRADO DE ENCOFRADO Y DESENCOFRADO</t>
   </si>
   <si>
-    <t>Criterio (lamina DA-02): se encofran las dos caras interiores de los muros, las dos caras exteriores en toda la altura del cajon (losa de fondo + muro + losa superior) y el fondo de la losa superior (ancho interior b). La losa de fondo se vacia sobre el solado y la cara superior de la losa queda libre (acabado).</t>
+    <t>Criterio (laminas DPLV-21 y DPLV-22): se encofran las dos caras interiores de los muros, las dos caras exteriores en toda la altura del cajon (losa de fondo + muro + losa superior) y el fondo de la losa superior (ancho interior b). La losa de fondo se vacia sobre el solado y la cara superior de la losa queda libre (acabado).</t>
   </si>
   <si>
     <t>ANCHO INT. b (m)</t>
@@ -2410,7 +2410,7 @@
     <t>TOTAL ENCOFRADO (m2)</t>
   </si>
   <si>
-    <t>DP-04 (secciones), DA-02 (areas por metro)</t>
+    <t>DPLV-21 y DPLV-22 (secciones y areas por metro)</t>
   </si>
   <si>
     <t>RESUMEN PARA LA PLANILLA GENERAL (partida 01.04.04.04.04)</t>
@@ -2419,7 +2419,7 @@
     <t>COLECTOR PLUVIAL FRONTAL - METRADO DE ACERO DE REFUERZO fy=4200 kg/cm2</t>
   </si>
   <si>
-    <t>Criterio (laminas DP-04 y DP-08, norma E.060 14.3.4): el tramo normal lleva un solo marco cerrado en el eje de muros y losas (perimetro = 2 x (ancho ext. - e) + 2 x (e fondo/2 + h + e losa/2) + ganchos); el cruce de camiones cisterna lleva marco exterior + marco interior de 1/2" (perimetros con recubrimiento 0.04). Barras longitudinales 3/8" en cada marco, con traslape de 0.40 cada 9.00 m. Peso: 3/8" = 0.56 kg/m, 1/2" = 0.994 kg/m.</t>
+    <t>Criterio (laminas DPLV-21 y DPLV-22, norma E.060 14.3.4): el tramo normal lleva un solo marco cerrado en el eje de muros y losas (perimetro = 2 x (ancho ext. - e) + 2 x (e fondo/2 + h + e losa/2) + ganchos); el cruce de camiones cisterna lleva marco exterior + marco interior de 1/2" (perimetros con recubrimiento 0.04). Barras longitudinales 3/8" en cada marco, con traslape de 0.40 cada 9.00 m. Peso: 3/8" = 0.56 kg/m, 1/2" = 0.994 kg/m.</t>
   </si>
   <si>
     <t>ESPAC. MARCOS s (m)</t>
@@ -2464,10 +2464,10 @@
     <t>TOTAL (kg)</t>
   </si>
   <si>
-    <t>DP-04 (seccion S-01), DP-08 (cuadro de doblado), DA-03</t>
-  </si>
-  <si>
-    <t>DP-04 (seccion S-02 a S-08), DP-08 (cuadro de doblado), DA-03</t>
+    <t>DPLV-21 (seccion S-01; armadura)</t>
+  </si>
+  <si>
+    <t>DPLV-21 y DPLV-22 (secciones S-02 a S-08; armadura)</t>
   </si>
   <si>
     <t>DIAM.</t>
@@ -2497,7 +2497,7 @@
     <t>recta</t>
   </si>
   <si>
-    <t>DP-06B, DD-01: 2 barras de 1/2" por lado, L = 1.40</t>
+    <t>DPLV-23, DPLV-27: 2 barras de 1/2" por lado, L = 1.40</t>
   </si>
   <si>
     <t>Parrilla de la tapa de concreto</t>
@@ -2539,7 +2539,7 @@
     <t>Registro en la losa del colector; empalme cuneta Eje 09</t>
   </si>
   <si>
-    <t>DP-01, DP-06B</t>
+    <t>DPLV-17, DPLV-23</t>
   </si>
   <si>
     <t>RV-02</t>
@@ -2647,7 +2647,7 @@
     <t>Juntas de dilatacion cada 4.00 m entre 0+004.00 y 0+104.00</t>
   </si>
   <si>
-    <t>DP-01; DP-02 (juntas en el perfil); DD-03; perimetro de la seccion</t>
+    <t>DPLV-17; DPLV-18 (juntas en el perfil); DPLV-29; perimetro de la seccion</t>
   </si>
   <si>
     <t>TOTAL JUNTA DE DILATACION (m)</t>
@@ -2656,13 +2656,13 @@
     <t>Contacto del colector con el muro este de la caja CL (perimetro de la seccion)</t>
   </si>
   <si>
-    <t>EMPALME DE CUNETA AL COLECTOR (ventana 0.40 x H en el muro lado predio, caida libre y registro encima) - laminas DP-06C y DD-04</t>
+    <t>EMPALME DE CUNETA AL COLECTOR (ventana 0.40 x H en el muro lado predio, caida libre y registro encima) - laminas DPLV-24 y DPLV-30</t>
   </si>
   <si>
     <t>Cuneta Eje 09 (registro RV-01)</t>
   </si>
   <si>
-    <t>DP-06C (cuadro de empalmes); DP-01</t>
+    <t>DPLV-24 (cuadro de empalmes); DPLV-17</t>
   </si>
   <si>
     <t>Cuneta Eje 08 (registro RV-03)</t>
@@ -2677,7 +2677,7 @@
     <t>TOTAL EMPALMES (und)</t>
   </si>
   <si>
-    <t>Nota: la cuneta del Eje 01 no entra al colector: cae directamente a la caja CL por una ventana en su muro norte (DP-07); esa ventana y la del muro este (llegada del colector) se dejan en la caja CL del expediente del Hogar de Refugio. Las cunetas se acortan hasta el muro (hoja CUNETAS - LLEGADA AL COLECTOR).</t>
+    <t>Nota: la cuneta del Eje 01 no entra al colector: cae directamente a la caja CL por una ventana en su muro norte (DPLV-25); esa ventana y la del muro este (llegada del colector) se dejan en la caja CL del expediente del Hogar de Refugio. Las cunetas se acortan hasta el muro (hoja CUNETAS - LLEGADA AL COLECTOR).</t>
   </si>
   <si>
     <t>COLECTOR PLUVIAL FRONTAL - DESGLOSE DE INSUMOS POR PARTIDA</t>
@@ -2857,7 +2857,7 @@
     <t>Desagregado por componente: ver hoja DESAGREGADO TAPA REGISTRO</t>
   </si>
   <si>
-    <t>Laminas DP-01, DP-02, DP-06C, DP-07 y DD-03. Junta de dilatacion de 1" cada 4.00 m en todo el perimetro de la seccion (tecnopor de 1" en todo el perimetro + sellador asfaltico RC-250 con arena de 1" x 2" en la cara expuesta, EG-2013 MTC). A ambos lados del colector hay terreno natural (sin piso): no lleva junta longitudinal; la losa superior sirve de vereda. Junta de tecnopor de 1" con sellador asfaltico en el contacto con la caja CL. Empalme de cada cuneta por ventana en el muro lado predio con caida libre al fondo (sin dintel adicional).</t>
+    <t>Laminas DPLV-17, DPLV-18, DPLV-24, DPLV-25 y DPLV-29. Junta de dilatacion de 1" cada 4.00 m en todo el perimetro de la seccion (tecnopor de 1" en todo el perimetro + sellador asfaltico RC-250 con arena de 1" x 2" en la cara expuesta, EG-2013 MTC). A ambos lados del colector hay terreno natural (sin piso): no lleva junta longitudinal; la losa superior sirve de vereda. Junta de tecnopor de 1" con sellador asfaltico en el contacto con la caja CL. Empalme de cada cuneta por ventana en el muro lado predio con caida libre al fondo (sin dintel adicional).</t>
   </si>
   <si>
     <t>JUNTA DE DILATACION e=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR (perimetro = 2 x ancho exterior + 2 x (e fondo + h max + e losa))</t>
@@ -2869,10 +2869,10 @@
     <t>Bordes de la losa: terreno natural a ambos lados (sin piso): no lleva junta</t>
   </si>
   <si>
-    <t>DP-04 y DD-03</t>
-  </si>
-  <si>
-    <t>DP-07 y DD-03: tecnopor y sellador en todo el contacto colector - CL</t>
+    <t>DPLV-21, DPLV-22 y DPLV-29</t>
+  </si>
+  <si>
+    <t>DPLV-25 y DPLV-29: tecnopor y sellador en todo el contacto colector - CL</t>
   </si>
   <si>
     <t>TOTAL JUNTA CON LA CAJA CL (m)</t>
@@ -2898,7 +2898,7 @@
     <t>2. Longitud por junta = 2 x altura del muro (area del muro / longitud del eje, hoja CONCRETO EN CUNETAS) + ancho interior del fondo 0.40 m.</t>
   </si>
   <si>
-    <t>3. Junta e = 1" (0.0254 m): tecnopor de 1" en todo el espesor y sellador asfaltico (RC-250 + arena) en la cara interior; se mide en metros lineales de junta sellada. Detalle en la lamina DJ-01.</t>
+    <t>3. Junta e = 1" (0.0254 m): tecnopor de 1" en todo el espesor y sellador asfaltico (RC-250 + arena) en la cara interior; se mide en metros lineales de junta sellada. Detalle en la lamina DPLV-31.</t>
   </si>
   <si>
     <t>01.04.04.04.01 CONCRETO f'c=210 PARA COLECTOR - losa de fondo</t>
@@ -3444,22 +3444,22 @@
     <t>ANALISIS DE COSTO UNITARIO - JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR</t>
   </si>
   <si>
-    <t>Partida de Delphin 01.04.04.06.01 JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR (metrado 01.04.04.06.01, hoja COLECTOR JUNTAS Y EMPALMES). Se mide por metro de junta a lo largo del perimetro de la seccion. Cantidades de la lamina DD-03: plancha de tecnopor de 1" en toda la seccion y sellador asfaltico 1" x 2" (asfalto liquido RC-250 + arena gruesa) en las caras interiores y en la cara superior (EG-2013 MTC, 510). Celda amarilla = dato; verde = formula. Precios sin IGV.</t>
-  </si>
-  <si>
-    <t>1. CANTIDADES POR METRO DE JUNTA (lamina DD-03 y hoja COLECTOR JUNTAS Y EMPALMES)</t>
-  </si>
-  <si>
-    <t>COLECTOR JUNTAS Y EMPALMES fila 11; DD-03 A</t>
+    <t>Partida de Delphin 01.04.04.06.01 JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ASFALTICO EN COLECTOR (metrado 01.04.04.06.01, hoja COLECTOR JUNTAS Y EMPALMES). Se mide por metro de junta a lo largo del perimetro de la seccion. Cantidades de la lamina DPLV-29: plancha de tecnopor de 1" en toda la seccion y sellador asfaltico 1" x 2" (asfalto liquido RC-250 + arena gruesa) en las caras interiores y en la cara superior (EG-2013 MTC, 510). Celda amarilla = dato; verde = formula. Precios sin IGV.</t>
+  </si>
+  <si>
+    <t>1. CANTIDADES POR METRO DE JUNTA (lamina DPLV-29 y hoja COLECTOR JUNTAS Y EMPALMES)</t>
+  </si>
+  <si>
+    <t>COLECTOR JUNTAS Y EMPALMES fila 11; DPLV-29 A</t>
   </si>
   <si>
     <t>Numero de juntas de dilatacion (cada 4.00 m)</t>
   </si>
   <si>
-    <t>COLECTOR JUNTAS Y EMPALMES fila 11; DD-03 E</t>
-  </si>
-  <si>
-    <t>DD-03, cuadro de componentes</t>
+    <t>COLECTOR JUNTAS Y EMPALMES fila 11; DPLV-29 E</t>
+  </si>
+  <si>
+    <t>DPLV-29, cuadro de componentes</t>
   </si>
   <si>
     <t>Tecnopor por metro de junta (area neta)</t>
@@ -3489,7 +3489,7 @@
     <t>Seccion del sellador 1" x 2" (0.0254 x 0.0508)</t>
   </si>
   <si>
-    <t>DD-03 B; EG-2013 MTC, Seccion 510</t>
+    <t>DPLV-29 B; EG-2013 MTC, Seccion 510</t>
   </si>
   <si>
     <t>Mezcla de sellador por metro de junta</t>
@@ -3582,13 +3582,13 @@
     <t>ANALISIS DE COSTO UNITARIO - JUNTA E=1" CON TECNOPOR Y SELLADOR ASFALTICO ENTRE COLECTOR Y CAJA CL</t>
   </si>
   <si>
-    <t>Partida de Delphin 01.04.04.06.02 JUNTA E=1" CON TECNOPOR Y SELLADOR ASFALTICO ENTRE COLECTOR Y CAJA CL (metrado 01.04.04.06.02, hoja COLECTOR JUNTAS Y EMPALMES). Se mide por metro de junta a lo largo del perimetro de la seccion, en el contacto del colector con el muro este de la caja CL. Cantidades de la lamina DD-03: plancha de tecnopor de 1" en toda la seccion y sellador asfaltico 1" x 2" (RC-250 + arena) en las caras interiores y en la cara superior. A ambos lados del colector hay terreno natural: no lleva junta longitudinal. Celda amarilla = dato; verde = formula. Precios sin IGV.</t>
+    <t>Partida de Delphin 01.04.04.06.02 JUNTA E=1" CON TECNOPOR Y SELLADOR ASFALTICO ENTRE COLECTOR Y CAJA CL (metrado 01.04.04.06.02, hoja COLECTOR JUNTAS Y EMPALMES). Se mide por metro de junta a lo largo del perimetro de la seccion, en el contacto del colector con el muro este de la caja CL. Cantidades de la lamina DPLV-29: plancha de tecnopor de 1" en toda la seccion y sellador asfaltico 1" x 2" (RC-250 + arena) en las caras interiores y en la cara superior. A ambos lados del colector hay terreno natural: no lleva junta longitudinal. Celda amarilla = dato; verde = formula. Precios sin IGV.</t>
   </si>
   <si>
     <t>Perimetro de la seccion en el contacto con la caja CL: 2 x 0.90 + 2 x (0.15 + 1.17 + 0.10)</t>
   </si>
   <si>
-    <t>COLECTOR JUNTAS Y EMPALMES fila 16; DD-03</t>
+    <t>COLECTOR JUNTAS Y EMPALMES fila 16; DPLV-29</t>
   </si>
   <si>
     <t>Numero de juntas en el contacto con la caja CL</t>
@@ -3618,7 +3618,7 @@
     <t>DESAGREGADO DE LA PARTIDA 01.04.03.04.03.04 - LLORADERO DE TUBERIA PVC Ø3" C/FILTRO DE GRAVA Y GEOTEXTIL @1.50 m</t>
   </si>
   <si>
-    <t>La partida se mide por unidad de lloradero. A: ubicacion y numero, de la hoja METRADO LLORADEROS (muros de cuneta colindantes con area verde, medidos en la planta general de drenaje; un lloradero cada 1.50 m). B: componentes de un lloradero segun las laminas DL-01 y DL-02 (tubo PVC-U Ø 3" de 0.30 m con 8 perforaciones Ø 3/8", filtro de grava de 0.30 x 0.30 x 0.30 m forrado con geotextil no tejido) por el numero de lloraderos. Celda amarilla = dato; verde = formula.</t>
+    <t>La partida se mide por unidad de lloradero. A: ubicacion y numero, de la hoja METRADO LLORADEROS (muros de cuneta colindantes con area verde, medidos en la planta general de drenaje; un lloradero cada 1.50 m). B: componentes de un lloradero segun las laminas DPLV-34 y DPLV-35 (tubo PVC-U Ø 3" de 0.30 m con 8 perforaciones Ø 3/8", filtro de grava de 0.30 x 0.30 x 0.30 m forrado con geotextil no tejido) por el numero de lloraderos. Celda amarilla = dato; verde = formula.</t>
   </si>
   <si>
     <t>A. UBICACION Y NUMERO DE LLORADEROS (hoja METRADO LLORADEROS)</t>
@@ -3639,31 +3639,31 @@
     <t>TOTAL (und de la partida)</t>
   </si>
   <si>
-    <t>B. DATOS DEL DETALLE (laminas DL-01 y DL-02)</t>
+    <t>B. DATOS DEL DETALLE (laminas DPLV-34 y DPLV-35)</t>
   </si>
   <si>
     <t>Lado del filtro localizado (cubo de grava forrado con geotextil)</t>
   </si>
   <si>
-    <t>DL-02 A: filtro 0.30 x 0.30 x 0.30 m</t>
+    <t>DPLV-35 A: filtro 0.30 x 0.30 x 0.30 m</t>
   </si>
   <si>
     <t>Longitud del tubo PVC-U Ø 3" por lloradero</t>
   </si>
   <si>
-    <t>DL-02 B: 0.10 en el muro + 0.20 perforado dentro del filtro</t>
+    <t>DPLV-35 B: 0.10 en el muro + 0.20 perforado dentro del filtro</t>
   </si>
   <si>
     <t>Perforaciones Ø 3/8" por fila</t>
   </si>
   <si>
-    <t>DL-02 B: 4 perforaciones @0.05 por fila</t>
+    <t>DPLV-35 B: 4 perforaciones @0.05 por fila</t>
   </si>
   <si>
     <t>Filas de perforaciones</t>
   </si>
   <si>
-    <t>DL-02 B: 2 filas a 120 grados, simetricas respecto al fondo</t>
+    <t>DPLV-35 B: 2 filas a 120 grados, simetricas respecto al fondo</t>
   </si>
   <si>
     <t>Desperdicio de grava (acomodo y perdidas)</t>
@@ -3675,13 +3675,13 @@
     <t>Traslapes del geotextil</t>
   </si>
   <si>
-    <t>DL-01 etapa 3: traslape de 0.10 m al cerrar el filtro</t>
+    <t>DPLV-34 etapa 3: traslape de 0.10 m al cerrar el filtro</t>
   </si>
   <si>
     <t>Mortero 1:3 de sellado alrededor del tubo</t>
   </si>
   <si>
-    <t>anillo de 0.02 m en las dos caras del muro (DL-02)</t>
+    <t>anillo de 0.02 m en las dos caras del muro (DPLV-35)</t>
   </si>
   <si>
     <t>C. COMPONENTES DE UN LLORADERO Y TOTAL DE LA PARTIDA</t>
@@ -3696,34 +3696,34 @@
     <t>Tubo PVC-U Ø 3" para desague (NTP 399.003)</t>
   </si>
   <si>
-    <t>DL-02 B; sale de tubos de 3 m (10 lloraderos por tubo)</t>
+    <t>DPLV-35 B; sale de tubos de 3 m (10 lloraderos por tubo)</t>
   </si>
   <si>
     <t>Perforaciones Ø 3/8" en el tramo dentro del filtro</t>
   </si>
   <si>
-    <t>DL-02 B</t>
+    <t>DPLV-35 B</t>
   </si>
   <si>
     <t>Excavacion local del hueco del filtro (lado^3)</t>
   </si>
   <si>
-    <t>DL-01 etapa 1; incluida en la mano de obra del ACU</t>
+    <t>DPLV-34 etapa 1; incluida en la mano de obra del ACU</t>
   </si>
   <si>
     <t>Grava filtrante (ripio) 20 a 40 mm: lado^3 + desperdicio</t>
   </si>
   <si>
-    <t>DL-01 etapa 2; DL-02 A</t>
+    <t>DPLV-34 etapa 2; DPLV-35 A</t>
   </si>
   <si>
     <t>Geotextil no tejido clase 2: 6 caras del cubo + traslapes</t>
   </si>
   <si>
-    <t>DL-01 etapa 3; DL-02 A</t>
-  </si>
-  <si>
-    <t>DL-02</t>
+    <t>DPLV-34 etapa 3; DPLV-35 A</t>
+  </si>
+  <si>
+    <t>DPLV-35</t>
   </si>
   <si>
     <t>D. CONTROL CON EL RESUMEN</t>
@@ -3738,7 +3738,7 @@
     <t>ANALISIS DE COSTO UNITARIO - LLORADERO DE TUBERIA PVC Ø3" C/FILTRO DE GRAVA Y GEOTEXTIL @1.50 m</t>
   </si>
   <si>
-    <t>Partida de Delphin 01.04.03.04.03.04 LLORADERO DE TUBERIA PVC Ø3" C/FILTRO DE GRAVA Y GEOTEXTIL @1.50 m (CUNETA COLINDANTE CON AREA VERDE) (metrado: hojas METRADO LLORADEROS y DESAGREGADO LLORADEROS). Cantidades por lloradero de las laminas DL-01 y DL-02: tubo PVC-U Ø 3" de 0.30 m con 8 perforaciones Ø 3/8", filtro de grava de 0.30 x 0.30 x 0.30 m forrado con geotextil no tejido y mortero 1:3 de sellado. Mano de obra de la hoja COSTO HORA HOMBRE 2026. Celda amarilla = dato; verde = formula. Precios sin IGV.</t>
+    <t>Partida de Delphin 01.04.03.04.03.04 LLORADERO DE TUBERIA PVC Ø3" C/FILTRO DE GRAVA Y GEOTEXTIL @1.50 m (CUNETA COLINDANTE CON AREA VERDE) (metrado: hojas METRADO LLORADEROS y DESAGREGADO LLORADEROS). Cantidades por lloradero de las laminas DPLV-34 y DPLV-35: tubo PVC-U Ø 3" de 0.30 m con 8 perforaciones Ø 3/8", filtro de grava de 0.30 x 0.30 x 0.30 m forrado con geotextil no tejido y mortero 1:3 de sellado. Mano de obra de la hoja COSTO HORA HOMBRE 2026. Celda amarilla = dato; verde = formula. Precios sin IGV.</t>
   </si>
   <si>
     <t>1. CANTIDADES POR LLORADERO (hoja DESAGREGADO LLORADEROS)</t>
@@ -3843,31 +3843,31 @@
     <t>DESAGREGADO LLORADEROS fila 45</t>
   </si>
   <si>
-    <t>DESAGREGADO LLORADEROS fila 59 (DL-02 B)</t>
-  </si>
-  <si>
-    <t>DESAGREGADO LLORADEROS fila 62 (DL-02 A)</t>
-  </si>
-  <si>
-    <t>DESAGREGADO LLORADEROS fila 63 (DL-01 etapa 3)</t>
-  </si>
-  <si>
-    <t>DESAGREGADO LLORADEROS fila 64 (DL-02)</t>
+    <t>DESAGREGADO LLORADEROS fila 59 (DPLV-35 B)</t>
+  </si>
+  <si>
+    <t>DESAGREGADO LLORADEROS fila 62 (DPLV-35 A)</t>
+  </si>
+  <si>
+    <t>DESAGREGADO LLORADEROS fila 63 (DPLV-34 etapa 3)</t>
+  </si>
+  <si>
+    <t>DESAGREGADO LLORADEROS fila 64 (DPLV-35)</t>
   </si>
   <si>
     <t>Borde engrosado de la abertura: perimetro (solo los 2 lados transversales, entre muros)</t>
   </si>
   <si>
-    <t>Lamina DP-06B: 2 x b; b = 0.60 es menor que la abertura de 0.70, en los lados largos el asiento es la cabeza del muro</t>
-  </si>
-  <si>
-    <t>REGISTROS DE LIMPIEZA EN LA LOSA DEL COLECTOR - lamina DP-06B (borde engrosado 0.15 x 0.10 solo en los 2 lados transversales, entre muros: en los lados largos la abertura apoya en la cabeza de los muros; descuento de la abertura 0.70 x 0.70 en la losa superior)</t>
+    <t>Lamina DPLV-23: 2 x b; b = 0.60 es menor que la abertura de 0.70, en los lados largos el asiento es la cabeza del muro</t>
+  </si>
+  <si>
+    <t>REGISTROS DE LIMPIEZA EN LA LOSA DEL COLECTOR - lamina DPLV-23 (borde engrosado 0.15 x 0.10 solo en los 2 lados transversales, entre muros: en los lados largos la abertura apoya en la cabeza de los muros; descuento de la abertura 0.70 x 0.70 en la losa superior)</t>
   </si>
   <si>
     <t>Registros RV-01 a RV-11: borde engrosado de la abertura (2 lados, entre muros)</t>
   </si>
   <si>
-    <t>DP-06B, DD-01: 2 x 0.60 m por registro, en los 11 registros</t>
+    <t>DPLV-23, DPLV-27: 2 x 0.60 m por registro, en los 11 registros</t>
   </si>
   <si>
     <t>Bordes engrosados de abertura de registros RV-01 a RV-11 (2 lados, entre muros)</t>
@@ -3876,13 +3876,13 @@
     <t>Lado del rebaje de asiento de la tapa en la losa (0.70 x 0.70 x 0.08)</t>
   </si>
   <si>
-    <t>Lamina DP-06B rev. 02 (tapa ciega)</t>
+    <t>Lamina DPLV-23 (tapa ciega)</t>
   </si>
   <si>
     <t>Luz libre del registro bajo el rebaje (0.60 x 0.60)</t>
   </si>
   <si>
-    <t>Lamina DP-06B rev. 02</t>
+    <t>Lamina DPLV-23</t>
   </si>
   <si>
     <t>Perimetro del encofrado lateral de la tapa (4 x 0.68)</t>
@@ -3900,10 +3900,10 @@
     <t>Bisel de los cantos superiores de la tapa</t>
   </si>
   <si>
-    <t>Lamina DP-06B rev. 02 (tapa ciega de concreto armado)</t>
-  </si>
-  <si>
-    <t>Lamina DP-06B rev. 02 (= profundidad del rebaje)</t>
+    <t>Lamina DPLV-23 (tapa ciega de concreto armado)</t>
+  </si>
+  <si>
+    <t>Lamina DPLV-23 (= profundidad del rebaje)</t>
   </si>
   <si>
     <t>Asas de izaje de la tapa (en cajuelas)</t>
@@ -3912,10 +3912,10 @@
     <t>1/2" liso</t>
   </si>
   <si>
-    <t>DP-06B rev. 02: 2 asas de fierro liso 1/2" por tapa, desarrollo 0.50</t>
-  </si>
-  <si>
-    <t>DP-06B rev. 02: 7 + 7 barras de 3/8" @0.10, L = 0.62</t>
+    <t>DPLV-23: 2 asas de fierro liso 1/2" por tapa, desarrollo 0.50</t>
+  </si>
+  <si>
+    <t>DPLV-23: 7 + 7 barras de 3/8" @0.10, L = 0.62</t>
   </si>
   <si>
     <t>ACERO DE REFUERZO EN TAPAS, BORDES Y ASAS</t>
@@ -3930,7 +3930,7 @@
     <t>TAPA DE REGISTRO CIEGA DE CONCRETO ARMADO 0.68x0.68x0.08 (vaciada aparte en obra)</t>
   </si>
   <si>
-    <t>DP-06B rev. 02</t>
+    <t>DPLV-23</t>
   </si>
   <si>
     <t>ENCOFRADO LATERAL DE LA TAPA (molde de madera)</t>
@@ -3945,7 +3945,7 @@
     <t>hoja COLECTOR ACERO</t>
   </si>
   <si>
-    <t>DP-06B rev. 02; COLECTOR ACERO</t>
+    <t>DPLV-23; COLECTOR ACERO</t>
   </si>
   <si>
     <t>ASIENTO DE LA TAPA: REBAJE DE CONCRETO 0.70 x 0.70 x 0.08 EN LA LOSA</t>
@@ -3954,13 +3954,13 @@
     <t>1 por registro (concreto incluido en la losa)</t>
   </si>
   <si>
-    <t>DP-06B rev. 02; COLECTOR CONCRETO</t>
+    <t>DPLV-23; COLECTOR CONCRETO</t>
   </si>
   <si>
     <t>COLOCACION DE LA TAPA EN EL REBAJE (izaje con las asas)</t>
   </si>
   <si>
-    <t>Lamina DP-01 (ubicacion) y DP-06B rev. 02 (detalle): tapa ciega de concreto armado 0.68 x 0.68 x 0.08, vaciada aparte en obra, con 2 asas de fierro liso 1/2", apoyada en un rebaje de concreto de 0.70 x 0.70 x 0.08 de la losa (luz libre 0.60 x 0.60). Sin marco ni contramarco metalico.</t>
+    <t>Lamina DPLV-17 (ubicacion) y DPLV-23 (detalle): tapa ciega de concreto armado 0.68 x 0.68 x 0.08, vaciada aparte en obra, con 2 asas de fierro liso 1/2", apoyada en un rebaje de concreto de 0.70 x 0.70 x 0.08 de la losa (luz libre 0.60 x 0.60). Sin marco ni contramarco metalico.</t>
   </si>
   <si>
     <t>01.04.04.05.01 TAPA DE REGISTRO: encofrado lateral de la tapa (molde de madera, 6 usos)</t>
@@ -4092,7 +4092,7 @@
     <t>Tapa ciega de concreto f'c=210: 0.68 x 0.68 x 0.08</t>
   </si>
   <si>
-    <t>lamina DP-06B rev. 02</t>
+    <t>lamina DPLV-23</t>
   </si>
   <si>
     <t>ENCOFRADO</t>
@@ -4119,16 +4119,16 @@
     <t>Acero en tapas, asas y bordes</t>
   </si>
   <si>
-    <t>No hay angulos, soldadura ni pintura: la tapa es ciega de concreto armado (lamina DP-06B rev. 02). El rebaje de asiento y el borde engrosado de la abertura se metran con el concreto de la losa del colector (hoja COLECTOR CONCRETO).</t>
-  </si>
-  <si>
-    <t>Lamina DP-06B rev. 02: agarre 0.15 + 2 patas de 0.02 + 2 ganchos de 0.15 (0.49, se toma 0.50)</t>
+    <t>No hay angulos, soldadura ni pintura: la tapa es ciega de concreto armado (lamina DPLV-23). El rebaje de asiento y el borde engrosado de la abertura se metran con el concreto de la losa del colector (hoja COLECTOR CONCRETO).</t>
+  </si>
+  <si>
+    <t>Lamina DPLV-23: agarre 0.15 + 2 patas de 0.02 + 2 ganchos de 0.15 (0.49, se toma 0.50)</t>
   </si>
   <si>
     <t>ACERO DE REFUERZO fy=4200 kg/cm2 EN TAPAS, BORDES Y ASAS</t>
   </si>
   <si>
-    <t>REGISTROS DE LIMPIEZA Y TAPAS - laminas DP-06B, DD-01 y DD-02: refuerzo de borde de la abertura, parrilla de la tapa, asas de la tapa ciega (cantidad de registros de la hoja COLECTOR REGISTROS Y TAPAS)</t>
+    <t>REGISTROS DE LIMPIEZA Y TAPAS - laminas DPLV-23, DPLV-27 y DPLV-28: refuerzo de borde de la abertura, parrilla de la tapa, asas de la tapa ciega (cantidad de registros de la hoja COLECTOR REGISTROS Y TAPAS)</t>
   </si>
 </sst>
 </file>
@@ -25753,7 +25753,7 @@
       </c>
       <c r="G11" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F10</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H11" s="217"/>
     </row>
@@ -25780,7 +25780,7 @@
       </c>
       <c r="G12" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F11</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H12" s="217"/>
     </row>
@@ -25807,7 +25807,7 @@
       </c>
       <c r="G13" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F12</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H13" s="217"/>
     </row>
@@ -25834,7 +25834,7 @@
       </c>
       <c r="G14" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F13</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H14" s="217"/>
     </row>
@@ -25861,7 +25861,7 @@
       </c>
       <c r="G15" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F14</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H15" s="217"/>
     </row>
@@ -25888,7 +25888,7 @@
       </c>
       <c r="G16" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F15</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H16" s="217"/>
     </row>
@@ -25915,7 +25915,7 @@
       </c>
       <c r="G17" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F16</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H17" s="217"/>
     </row>
@@ -25942,7 +25942,7 @@
       </c>
       <c r="G18" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F17</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H18" s="217"/>
     </row>
@@ -25969,7 +25969,7 @@
       </c>
       <c r="G19" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F18</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H19" s="217"/>
     </row>
@@ -25996,7 +25996,7 @@
       </c>
       <c r="G20" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F19</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H20" s="217"/>
     </row>
@@ -26023,7 +26023,7 @@
       </c>
       <c r="G21" s="111" t="str">
         <f>+'COLECTOR REGISTROS Y TAPAS'!F20</f>
-        <v>DP-01, DP-06B</v>
+        <v>DPLV-17, DPLV-23</v>
       </c>
       <c r="H21" s="217"/>
     </row>

</xml_diff>